<commit_message>
pcbWay images to Order
</commit_message>
<xml_diff>
--- a/Manufacturing Files/devBoard BOM PCBWay.xlsx
+++ b/Manufacturing Files/devBoard BOM PCBWay.xlsx
@@ -5,12 +5,12 @@
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Documents\GitHub\Embedded-Systems-Instructor\Dev Board Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Documents\GitHub\Embedded-Systems-Instructor\Manufacturing Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5CB1A33-C797-4EA1-8D78-97F414B72344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9036DA-888F-4081-B82B-EBECCFA8CBEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Digikey" sheetId="4" r:id="rId1"/>
@@ -139,12 +139,6 @@
     <t>Microchips</t>
   </si>
   <si>
-    <t>PIC18F26K22-I/SS-ND</t>
-  </si>
-  <si>
-    <t>PIC18F26K22-I/SS</t>
-  </si>
-  <si>
     <t>TI</t>
   </si>
   <si>
@@ -343,9 +337,6 @@
     <t>Terminal Block</t>
   </si>
   <si>
-    <t>PIC 18F26K22</t>
-  </si>
-  <si>
     <t>Serial USB bridge</t>
   </si>
   <si>
@@ -514,9 +505,6 @@
     <t>IC1, IC4</t>
   </si>
   <si>
-    <t>PIC18F26K22</t>
-  </si>
-  <si>
     <t>LED6</t>
   </si>
   <si>
@@ -584,6 +572,18 @@
   </si>
   <si>
     <t>67-1359-1-ND</t>
+  </si>
+  <si>
+    <t>PIC 18F25K22</t>
+  </si>
+  <si>
+    <t>PIC18F25K22</t>
+  </si>
+  <si>
+    <t>PIC18F25K22-I/SS</t>
+  </si>
+  <si>
+    <t>PIC18F25K22-I/SS-ND</t>
   </si>
 </sst>
 </file>
@@ -1645,55 +1645,55 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>23</v>
@@ -1719,19 +1719,19 @@
     </row>
     <row r="4" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>23</v>
@@ -1757,19 +1757,19 @@
     </row>
     <row r="5" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>23</v>
@@ -1795,19 +1795,19 @@
     </row>
     <row r="6" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>23</v>
@@ -1833,19 +1833,19 @@
     </row>
     <row r="7" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>23</v>
@@ -1871,19 +1871,19 @@
     </row>
     <row r="8" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>23</v>
@@ -1909,19 +1909,19 @@
     </row>
     <row r="9" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>23</v>
@@ -1947,19 +1947,19 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>23</v>
@@ -1998,10 +1998,10 @@
     </row>
     <row r="12" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>3</v>
@@ -2036,19 +2036,19 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>13</v>
@@ -2073,19 +2073,19 @@
     </row>
     <row r="14" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>13</v>
@@ -2111,19 +2111,19 @@
     </row>
     <row r="15" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>13</v>
@@ -2149,19 +2149,19 @@
     </row>
     <row r="16" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>13</v>
@@ -2197,10 +2197,10 @@
     </row>
     <row r="18" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>18</v>
@@ -2209,7 +2209,7 @@
         <v>901200122</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>19</v>
@@ -2235,10 +2235,10 @@
     </row>
     <row r="19" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>18</v>
@@ -2247,7 +2247,7 @@
         <v>901200123</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>19</v>
@@ -2273,10 +2273,10 @@
     </row>
     <row r="20" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>18</v>
@@ -2285,7 +2285,7 @@
         <v>901200126</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>19</v>
@@ -2311,10 +2311,10 @@
     </row>
     <row r="21" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>20</v>
@@ -2323,7 +2323,7 @@
         <v>22288061</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>19</v>
@@ -2349,10 +2349,10 @@
     </row>
     <row r="22" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>2</v>
@@ -2387,22 +2387,22 @@
     </row>
     <row r="23" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G23" s="4">
         <v>0.35770000000000002</v>
@@ -2425,22 +2425,22 @@
     </row>
     <row r="24" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C24" s="3" t="s">
+      <c r="F24" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="G24" s="4">
         <v>8.2400000000000001E-2</v>
@@ -2463,10 +2463,10 @@
     </row>
     <row r="25" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>21</v>
@@ -2501,19 +2501,19 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="E26" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>12</v>
@@ -2548,19 +2548,19 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>100</v>
+        <v>177</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>31</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>33</v>
+        <v>179</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>32</v>
+        <v>180</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>25</v>
@@ -2585,22 +2585,22 @@
     </row>
     <row r="29" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G29" s="4">
         <v>1.9</v>
@@ -2623,10 +2623,10 @@
     </row>
     <row r="30" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>11</v>
@@ -2661,22 +2661,22 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G31" s="2">
         <v>0.05</v>
@@ -2698,22 +2698,22 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>31</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G32" s="2">
         <v>0.41</v>
@@ -2735,19 +2735,19 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>24</v>
@@ -2772,19 +2772,19 @@
     </row>
     <row r="34" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>22</v>
@@ -2810,10 +2810,10 @@
     </row>
     <row r="35" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>8</v>
@@ -2848,19 +2848,19 @@
     </row>
     <row r="36" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>17</v>
@@ -2886,19 +2886,19 @@
     </row>
     <row r="37" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>17</v>
@@ -2924,22 +2924,22 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G38" s="4">
         <v>0.36480000000000001</v>
@@ -2961,22 +2961,22 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G39" s="2">
         <v>0.8639</v>

</xml_diff>